<commit_message>
update seeder & template
</commit_message>
<xml_diff>
--- a/public/assets/template/gelanggang-template.xlsx
+++ b/public/assets/template/gelanggang-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ndejo\Documents\GitHub\simaps-ukasya\public\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FDBF414-5AA5-4209-BF56-041B5C7DA802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D50C9DA-0ACC-4BDA-B406-76AFB150B5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10245" windowHeight="10920" xr2:uid="{51F6D04B-38A7-4907-901E-8D2AF0D93E74}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="15375" windowHeight="7875" xr2:uid="{51F6D04B-38A7-4907-901E-8D2AF0D93E74}"/>
   </bookViews>
   <sheets>
     <sheet name="Lembar1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Nama</t>
   </si>
@@ -51,15 +51,9 @@
     <t>Jenis</t>
   </si>
   <si>
-    <t>Jumlah</t>
-  </si>
-  <si>
     <t>Arena A</t>
   </si>
   <si>
-    <t>suara.mp3</t>
-  </si>
-  <si>
     <t>Arena B</t>
   </si>
   <si>
@@ -69,7 +63,16 @@
     <t>Arena D</t>
   </si>
   <si>
-    <t>Arena E</t>
+    <t>audio.mp3</t>
+  </si>
+  <si>
+    <t>Tanding</t>
+  </si>
+  <si>
+    <t>Ganda</t>
+  </si>
+  <si>
+    <t>Regu</t>
   </si>
 </sst>
 </file>
@@ -140,12 +143,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -462,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A86521A1-DC6B-4F40-AA0D-147BEF52CF9B}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" style="1" bestFit="1" customWidth="1"/>
@@ -486,93 +492,62 @@
       <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1">
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1">
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="E3" s="1">
-        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="1">
-        <v>3</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" s="1">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>